<commit_message>
vault backup: 2026-05-18 12:03:01
</commit_message>
<xml_diff>
--- a/BWL/Übung/Übungen/UE07/UE07_Arbeitsblatt.xlsx
+++ b/BWL/Übung/Übungen/UE07/UE07_Arbeitsblatt.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="7.1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="7.2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="7.3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="7.7" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -18,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t>Produkt</t>
   </si>
@@ -81,17 +82,238 @@
   </si>
   <si>
     <t>Fixkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aufgabe 7.3</t>
+  </si>
+  <si>
+    <t>Verkaufspreis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stückkosten (zu Vollkosten)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable Stückkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geplante Absatzmenge 20xx</t>
+  </si>
+  <si>
+    <t>Fertigungszeit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapazität bei Normalarbeitszeit</t>
+  </si>
+  <si>
+    <t>Nebenrechnungen:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deckungsbeitrag / stück</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapazität pro Jahr (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kapazität pro Jahr (min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max. Produktionsmenge pro Jahr</t>
+  </si>
+  <si>
+    <t>Berechnung</t>
+  </si>
+  <si>
+    <t>Ergebnis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a) Break-Even-Menge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixkosten / Deckungsbeitrag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b) Deckungsumsatz (Umsatz am BEP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Break-Even-Menge * Verkaufspreis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c) Kapazitätsauslastung bei Kostendeckung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Break-Even-Menge / max. Produktionsmenge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d) Gewinn bei Planabsatzmenge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Planabsatzmenge * db - Fixkosten)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e) geplanter Umsatz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planabsatzmenge * Verkaufspreis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e) Umsatzrentabilität bei Planabsatzmenge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plangewinn / Planumsatz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f)  Gewinn bei Preisnachlass von Ums.rent.:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkaufsmenge: Planabsatzmenge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neuer Preis:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkaufspreis * (1-Umsatzrent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neuer Umsatz:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neuerPreis * Planabsatzmenge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neuer Deckungsbeitrag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neuerPreis - varKosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neuer Gewinn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planmenge*neuDB - Fixkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g) verkraftbarer Anstieg der variablen Kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a = PlanabsMeng * preis - Fixkosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verkraftbarer Anstieg auf C34 ohne Verlust</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a / PlanabsMeng</t>
+  </si>
+  <si>
+    <t>Erlöse/Stk</t>
+  </si>
+  <si>
+    <t>var.Kost/Stück</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fertigungszeit/Stück (min)</t>
+  </si>
+  <si>
+    <t>db/Stück</t>
+  </si>
+  <si>
+    <t>db/min</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D.h. Reihenfolge:</t>
+  </si>
+  <si>
+    <t>1.</t>
+  </si>
+  <si>
+    <t>2.</t>
+  </si>
+  <si>
+    <t>3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">120 Stück A1 müssen jedoch aufgrund des Vertrages produziert werden.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prod. Stück</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verwendete Zeit (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">db gesamt: db/stück * prod.Stück</t>
+  </si>
+  <si>
+    <t xml:space="preserve">db Gesamt:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">optimale Verteilung wäre:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">db Gesamt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dbGesamt1 (Aufgabe b)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dbGesamt0 (Aufgabe a)</t>
+  </si>
+  <si>
+    <t>Differenz:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strafe dürfte also 2400€ sein.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00\ [$€-407]"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="7">
     <font>
+      <sz val="11.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -118,13 +340,33 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="18">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="1" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -151,7 +393,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>167639</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="3151265" cy="1689734"/>
+    <xdr:ext cx="3151265" cy="1689733"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1828788549" name=""/>
@@ -185,9 +427,9 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>609599</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>51434</xdr:rowOff>
+      <xdr:rowOff>51433</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="3921732" cy="1283968"/>
+    <xdr:ext cx="3921732" cy="1283967"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1682100589" name=""/>
@@ -745,15 +987,15 @@
         <v>500000</v>
       </c>
       <c r="F15" s="2">
-        <f>E15/C15</f>
+        <f t="shared" ref="F15:F18" si="0">E15/C15</f>
         <v>25</v>
       </c>
       <c r="G15" s="3">
-        <f>D15-F15</f>
+        <f t="shared" ref="G15:G18" si="1">D15-F15</f>
         <v>5</v>
       </c>
       <c r="H15">
-        <f>G15*C15</f>
+        <f t="shared" ref="H15:H18" si="2">G15*C15</f>
         <v>100000</v>
       </c>
     </row>
@@ -771,15 +1013,15 @@
         <v>580000</v>
       </c>
       <c r="F16" s="2">
-        <f>E16/C16</f>
+        <f t="shared" si="0"/>
         <v>38.666666666666664</v>
       </c>
       <c r="G16" s="3">
-        <f>D16-F16</f>
+        <f t="shared" si="1"/>
         <v>1.3333333333333357</v>
       </c>
       <c r="H16">
-        <f>G16*C16</f>
+        <f t="shared" si="2"/>
         <v>20000.000000000036</v>
       </c>
     </row>
@@ -797,15 +1039,15 @@
         <v>100000</v>
       </c>
       <c r="F17" s="2">
-        <f>E17/C17</f>
+        <f t="shared" si="0"/>
         <v>5.5555555555555554</v>
       </c>
       <c r="G17" s="3">
-        <f>D17-F17</f>
+        <f t="shared" si="1"/>
         <v>4.4444444444444446</v>
       </c>
       <c r="H17">
-        <f>G17*C17</f>
+        <f t="shared" si="2"/>
         <v>80000</v>
       </c>
     </row>
@@ -823,15 +1065,15 @@
         <v>90000</v>
       </c>
       <c r="F18" s="2">
-        <f>E18/C18</f>
+        <f t="shared" si="0"/>
         <v>2.25</v>
       </c>
       <c r="G18" s="3">
-        <f>D18-F18</f>
+        <f t="shared" si="1"/>
         <v>2.75</v>
       </c>
       <c r="H18">
-        <f>G18*C18</f>
+        <f t="shared" si="2"/>
         <v>110000</v>
       </c>
     </row>
@@ -931,11 +1173,747 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col bestFit="1" min="1" max="1" style="4" width="40.90234375"/>
+    <col bestFit="1" min="2" max="2" style="4" width="40.04296875"/>
+    <col bestFit="1" min="3" max="3" style="4" width="15.25390625"/>
+    <col min="4" max="16384" style="4" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75">
+      <c r="A1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+    </row>
+    <row r="2" ht="14.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+    </row>
+    <row r="3" ht="14.25">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="6"/>
+    </row>
+    <row r="4" ht="14.25">
+      <c r="A4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="8">
+        <v>516</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="6"/>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="8">
+        <v>414</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="A6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="8">
+        <v>2536000</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="8">
+        <v>316</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="8">
+        <v>22000</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="6"/>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="A9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="8">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="6"/>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="A10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="8">
+        <v>600</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10" s="6"/>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="A13" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="8">
+        <f>B4-B7</f>
+        <v>200</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="6"/>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="10">
+        <f>B10*12</f>
+        <v>7200</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="10">
+        <f>B15*60</f>
+        <v>432000</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="A17" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="10">
+        <f>B16/B9</f>
+        <v>22268.041237113404</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="6"/>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="6"/>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="7">
+        <f>B6/B14</f>
+        <v>12680</v>
+      </c>
+      <c r="D20" s="7"/>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="8">
+        <f>C20*B4</f>
+        <v>6542880</v>
+      </c>
+      <c r="D21" s="7"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="12">
+        <f>C20/B17</f>
+        <v>0.56942592592592589</v>
+      </c>
+      <c r="D22" s="7"/>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="A23" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="8">
+        <f>(B8*B14)-B6</f>
+        <v>1864000</v>
+      </c>
+      <c r="D23" s="7"/>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="8">
+        <f>B8*B4</f>
+        <v>11352000</v>
+      </c>
+      <c r="D24" s="7"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="A25" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="12">
+        <f>C23/C24</f>
+        <v>0.164200140944327</v>
+      </c>
+      <c r="D25" s="7"/>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="7"/>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="A27" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="7"/>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="A28" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="13">
+        <f>B4*(1-C25)</f>
+        <v>431.27272727272725</v>
+      </c>
+      <c r="D28" s="7"/>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="A29" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" s="13">
+        <f>C28*B8</f>
+        <v>9488000</v>
+      </c>
+      <c r="D29" s="7"/>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="A30" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" s="13">
+        <f>C28-B7</f>
+        <v>115.27272727272725</v>
+      </c>
+      <c r="D30" s="7"/>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="A31" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" s="14">
+        <f>(B8*C30)-B6</f>
+        <v>-4.6566128730773926e-10</v>
+      </c>
+      <c r="D31" s="7"/>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="6"/>
+    </row>
+    <row r="33" ht="14.25">
+      <c r="A33" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" s="13">
+        <f>(B8*B4)-B6</f>
+        <v>8816000</v>
+      </c>
+      <c r="D33" s="6"/>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="A34" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="13">
+        <f>C33/B8</f>
+        <v>400.72727272727275</v>
+      </c>
+      <c r="D34" s="6"/>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="A36" s="7"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="6"/>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="A37" s="7"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="6"/>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="A38" s="7"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="6"/>
+    </row>
+    <row r="39" ht="14.25">
+      <c r="A39" s="7"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="6"/>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="A40" s="7"/>
+      <c r="B40" s="6"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="6"/>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="A41" s="7"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="6"/>
+    </row>
+    <row r="42" ht="14.25">
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+    </row>
+  </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="10.421875"/>
+    <col customWidth="1" min="3" max="3" width="12.421875"/>
+    <col customWidth="1" min="4" max="4" width="21.8515625"/>
+    <col bestFit="1" min="5" max="5" width="28.390625"/>
+    <col bestFit="1" min="9" max="9" width="11.83203125"/>
+  </cols>
+  <sheetData>
+    <row r="4" ht="14.25">
+      <c r="B4" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5">
+        <v>400</v>
+      </c>
+      <c r="D5">
+        <v>200</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <f>C5-D5</f>
+        <v>200</v>
+      </c>
+      <c r="G5">
+        <f>F5/E5</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="B6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6">
+        <v>350</v>
+      </c>
+      <c r="D6">
+        <v>250</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <f>C6-D6</f>
+        <v>100</v>
+      </c>
+      <c r="G6">
+        <f>F6/E6</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="B7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7">
+        <v>450</v>
+      </c>
+      <c r="D7">
+        <v>285</v>
+      </c>
+      <c r="E7">
+        <v>15</v>
+      </c>
+      <c r="F7">
+        <f>C7-D7</f>
+        <v>165</v>
+      </c>
+      <c r="G7">
+        <f>F7/E7</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="B11" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" s="1"/>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="B12" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="B14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="B16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="B18" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="B19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19">
+        <v>120</v>
+      </c>
+      <c r="D19">
+        <f>(C19*E5)/60</f>
+        <v>40</v>
+      </c>
+      <c r="E19">
+        <f>C19*F5</f>
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="B20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20">
+        <v>1800</v>
+      </c>
+      <c r="D20">
+        <f>(C20*E6)/60</f>
+        <v>150</v>
+      </c>
+      <c r="E20">
+        <f>C20*F6</f>
+        <v>180000</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="B21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21">
+        <f>(10*60)/15</f>
+        <v>40</v>
+      </c>
+      <c r="D21">
+        <v>10</v>
+      </c>
+      <c r="E21">
+        <f>C21*F7</f>
+        <v>6600</v>
+      </c>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" t="s">
+        <v>77</v>
+      </c>
+      <c r="E23">
+        <f>SUM(E19:E21)</f>
+        <v>210600</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="B26" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="B28" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="B29" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="6">
+        <v>0</v>
+      </c>
+      <c r="D29" s="6">
+        <v>0</v>
+      </c>
+      <c r="E29" s="6">
+        <f>F5*C29</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="17"/>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="B30" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="6">
+        <v>1800</v>
+      </c>
+      <c r="D30" s="6">
+        <f>(C30*E6)/60</f>
+        <v>150</v>
+      </c>
+      <c r="E30" s="6">
+        <f>F6*C30</f>
+        <v>180000</v>
+      </c>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="B31" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="6">
+        <f>(D31*60)/E7</f>
+        <v>200</v>
+      </c>
+      <c r="D31" s="6">
+        <v>50</v>
+      </c>
+      <c r="E31" s="6">
+        <f>F7*C31</f>
+        <v>33000</v>
+      </c>
+    </row>
+    <row r="33" ht="14.25">
+      <c r="D33" t="s">
+        <v>79</v>
+      </c>
+      <c r="E33">
+        <f>SUM(E29:E31)</f>
+        <v>213000</v>
+      </c>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="D37" t="s">
+        <v>80</v>
+      </c>
+      <c r="E37">
+        <f>E33</f>
+        <v>213000</v>
+      </c>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="D38" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38">
+        <f>E23</f>
+        <v>210600</v>
+      </c>
+    </row>
+    <row r="39" ht="14.25">
+      <c r="D39" t="s">
+        <v>82</v>
+      </c>
+      <c r="E39" s="16">
+        <f>E37-E38</f>
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="D41" t="s">
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="85" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-05-18 20:20:20
</commit_message>
<xml_diff>
--- a/BWL/Übung/Übungen/UE07/UE07_Arbeitsblatt.xlsx
+++ b/BWL/Übung/Übungen/UE07/UE07_Arbeitsblatt.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="7.1" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t>Produkt</t>
   </si>
@@ -156,10 +156,16 @@
     <t xml:space="preserve">Planabsatzmenge * Verkaufspreis</t>
   </si>
   <si>
+    <t xml:space="preserve">Umsatz ist natürlich ohne Ust - Ust und Vst werden</t>
+  </si>
+  <si>
     <t xml:space="preserve">e) Umsatzrentabilität bei Planabsatzmenge</t>
   </si>
   <si>
     <t xml:space="preserve">Plangewinn / Planumsatz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wo anders berechnet</t>
   </si>
   <si>
     <t xml:space="preserve">f)  Gewinn bei Preisnachlass von Ums.rent.:</t>
@@ -340,7 +346,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -358,6 +364,9 @@
     <xf fontId="3" fillId="0" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="10" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -393,7 +402,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>167639</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="3151265" cy="1689733"/>
+    <xdr:ext cx="3151265" cy="1689732"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="1828788549" name=""/>
@@ -427,7 +436,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>609599</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>51433</xdr:rowOff>
+      <xdr:rowOff>51432</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3921732" cy="1283967"/>
     <xdr:pic>
@@ -1398,7 +1407,7 @@
       <c r="A23" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="13" t="s">
         <v>42</v>
       </c>
       <c r="C23" s="8">
@@ -1419,23 +1428,29 @@
         <v>11352000</v>
       </c>
       <c r="D24" s="7"/>
+      <c r="E24" s="4" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="25" ht="14.25">
       <c r="A25" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C25" s="12">
         <f>C23/C24</f>
         <v>0.164200140944327</v>
       </c>
       <c r="D25" s="7"/>
+      <c r="E25" s="4" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="26" ht="14.25">
       <c r="A26" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1443,7 +1458,7 @@
     </row>
     <row r="27" ht="14.25">
       <c r="A27" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1451,12 +1466,12 @@
     </row>
     <row r="28" ht="14.25">
       <c r="A28" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="13">
+        <v>52</v>
+      </c>
+      <c r="C28" s="14">
         <f>B4*(1-C25)</f>
         <v>431.27272727272725</v>
       </c>
@@ -1464,12 +1479,12 @@
     </row>
     <row r="29" ht="14.25">
       <c r="A29" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C29" s="13">
+        <v>54</v>
+      </c>
+      <c r="C29" s="14">
         <f>C28*B8</f>
         <v>9488000</v>
       </c>
@@ -1477,12 +1492,12 @@
     </row>
     <row r="30" ht="14.25">
       <c r="A30" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C30" s="13">
+        <v>56</v>
+      </c>
+      <c r="C30" s="14">
         <f>C28-B7</f>
         <v>115.27272727272725</v>
       </c>
@@ -1490,12 +1505,12 @@
     </row>
     <row r="31" ht="14.25">
       <c r="A31" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31" s="14">
+        <v>58</v>
+      </c>
+      <c r="C31" s="15">
         <f>(B8*C30)-B6</f>
         <v>-4.6566128730773926e-10</v>
       </c>
@@ -1504,17 +1519,17 @@
     <row r="32" ht="14.25">
       <c r="A32" s="6"/>
       <c r="B32" s="6"/>
-      <c r="C32" s="15"/>
+      <c r="C32" s="16"/>
       <c r="D32" s="6"/>
     </row>
     <row r="33" ht="14.25">
       <c r="A33" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C33" s="13">
+        <v>60</v>
+      </c>
+      <c r="C33" s="14">
         <f>(B8*B4)-B6</f>
         <v>8816000</v>
       </c>
@@ -1522,12 +1537,12 @@
     </row>
     <row r="34" ht="14.25">
       <c r="A34" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C34" s="13">
+        <v>62</v>
+      </c>
+      <c r="C34" s="14">
         <f>C33/B8</f>
         <v>400.72727272727275</v>
       </c>
@@ -1605,28 +1620,28 @@
   </cols>
   <sheetData>
     <row r="4" ht="14.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="16" t="s">
+      <c r="C4" s="17" t="s">
         <v>63</v>
       </c>
+      <c r="D4" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>65</v>
+      </c>
       <c r="F4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" ht="14.25">
       <c r="B5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C5">
         <v>400</v>
@@ -1638,17 +1653,17 @@
         <v>20</v>
       </c>
       <c r="F5">
-        <f>C5-D5</f>
+        <f t="shared" ref="F5:F7" si="3">C5-D5</f>
         <v>200</v>
       </c>
       <c r="G5">
-        <f>F5/E5</f>
+        <f t="shared" ref="G5:G7" si="4">F5/E5</f>
         <v>10</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="B6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C6">
         <v>350</v>
@@ -1660,17 +1675,17 @@
         <v>5</v>
       </c>
       <c r="F6">
-        <f>C6-D6</f>
+        <f t="shared" si="3"/>
         <v>100</v>
       </c>
       <c r="G6">
-        <f>F6/E6</f>
+        <f t="shared" si="4"/>
         <v>20</v>
       </c>
     </row>
     <row r="7" ht="14.25">
       <c r="B7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C7">
         <v>450</v>
@@ -1682,98 +1697,98 @@
         <v>15</v>
       </c>
       <c r="F7">
-        <f>C7-D7</f>
+        <f t="shared" si="3"/>
         <v>165</v>
       </c>
       <c r="G7">
-        <f>F7/E7</f>
+        <f t="shared" si="4"/>
         <v>11</v>
       </c>
     </row>
     <row r="11" ht="14.25">
       <c r="B11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I11" s="1"/>
     </row>
     <row r="12" ht="14.25">
       <c r="B12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" ht="14.25">
       <c r="B13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" ht="14.25">
       <c r="B14" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="B16" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C18" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="E18" s="16" t="s">
+      <c r="C18" s="17" t="s">
         <v>76</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="19" ht="14.25">
       <c r="B19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C19">
         <v>120</v>
       </c>
       <c r="D19">
-        <f>(C19*E5)/60</f>
+        <f t="shared" ref="D19:D20" si="5">(C19*E5)/60</f>
         <v>40</v>
       </c>
       <c r="E19">
-        <f>C19*F5</f>
+        <f t="shared" ref="E19:E21" si="6">C19*F5</f>
         <v>24000</v>
       </c>
     </row>
     <row r="20" ht="14.25">
       <c r="B20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C20">
         <v>1800</v>
       </c>
       <c r="D20">
-        <f>(C20*E6)/60</f>
+        <f t="shared" si="5"/>
         <v>150</v>
       </c>
       <c r="E20">
-        <f>C20*F6</f>
+        <f t="shared" si="6"/>
         <v>180000</v>
       </c>
     </row>
     <row r="21" ht="14.25">
       <c r="B21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C21">
         <f>(10*60)/15</f>
@@ -1783,7 +1798,7 @@
         <v>10</v>
       </c>
       <c r="E21">
-        <f>C21*F7</f>
+        <f t="shared" si="6"/>
         <v>6600</v>
       </c>
     </row>
@@ -1792,7 +1807,7 @@
         <v>14</v>
       </c>
       <c r="D23" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E23">
         <f>SUM(E19:E21)</f>
@@ -1804,26 +1819,26 @@
         <v>16</v>
       </c>
       <c r="C26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="B28" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="E28" s="17" t="s">
         <v>78</v>
-      </c>
-    </row>
-    <row r="28" ht="14.25">
-      <c r="B28" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="29" ht="14.25">
       <c r="B29" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C29" s="6">
         <v>0</v>
@@ -1832,14 +1847,14 @@
         <v>0</v>
       </c>
       <c r="E29" s="6">
-        <f>F5*C29</f>
+        <f t="shared" ref="E29:E31" si="7">F5*C29</f>
         <v>0</v>
       </c>
-      <c r="I29" s="17"/>
+      <c r="I29" s="18"/>
     </row>
     <row r="30" ht="14.25">
       <c r="B30" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C30" s="6">
         <v>1800</v>
@@ -1849,13 +1864,13 @@
         <v>150</v>
       </c>
       <c r="E30" s="6">
-        <f>F6*C30</f>
+        <f t="shared" si="7"/>
         <v>180000</v>
       </c>
     </row>
     <row r="31" ht="14.25">
       <c r="B31" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C31" s="6">
         <f>(D31*60)/E7</f>
@@ -1865,13 +1880,13 @@
         <v>50</v>
       </c>
       <c r="E31" s="6">
-        <f>F7*C31</f>
+        <f t="shared" si="7"/>
         <v>33000</v>
       </c>
     </row>
     <row r="33" ht="14.25">
       <c r="D33" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E33">
         <f>SUM(E29:E31)</f>
@@ -1880,7 +1895,7 @@
     </row>
     <row r="37" ht="14.25">
       <c r="D37" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E37">
         <f>E33</f>
@@ -1889,7 +1904,7 @@
     </row>
     <row r="38" ht="14.25">
       <c r="D38" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E38">
         <f>E23</f>
@@ -1898,16 +1913,16 @@
     </row>
     <row r="39" ht="14.25">
       <c r="D39" t="s">
-        <v>82</v>
-      </c>
-      <c r="E39" s="16">
+        <v>84</v>
+      </c>
+      <c r="E39" s="17">
         <f>E37-E38</f>
         <v>2400</v>
       </c>
     </row>
     <row r="41" ht="14.25">
       <c r="D41" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>